<commit_message>
Add new stats/plots folders and files created by Python script
</commit_message>
<xml_diff>
--- a/Input_data/EST_All Countries_trad_eco_cal_2025-02-14_to_2025-02-25.xlsx
+++ b/Input_data/EST_All Countries_trad_eco_cal_2025-02-14_to_2025-02-25.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G393"/>
+  <dimension ref="A1:G397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3214,12 +3214,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>European Commission Winter Forecasts</t>
+          <t>ImportsJAN</t>
         </is>
       </c>
       <c r="D93" t="inlineStr"/>
@@ -3333,12 +3333,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>ImportsJAN</t>
+          <t>European Commission Winter Forecasts</t>
         </is>
       </c>
       <c r="D98" t="inlineStr"/>
@@ -3383,17 +3383,21 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>RBA Press Conference</t>
+          <t>Auto Production YoYJAN</t>
         </is>
       </c>
       <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr"/>
-      <c r="F100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>4.0%</t>
+        </is>
+      </c>
       <c r="G100" t="n">
         <v>2</v>
       </c>
@@ -3406,21 +3410,17 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Budget BalanceJAN</t>
+          <t>RBA Press Conference</t>
         </is>
       </c>
       <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr"/>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>TRY-150.0B</t>
-        </is>
-      </c>
+      <c r="F101" t="inlineStr"/>
       <c r="G101" t="n">
         <v>2</v>
       </c>
@@ -3438,14 +3438,14 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Auto Production YoYJAN</t>
+          <t>Budget BalanceJAN</t>
         </is>
       </c>
       <c r="D102" t="inlineStr"/>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>TRY-150.0B</t>
         </is>
       </c>
       <c r="G102" t="n">
@@ -3542,14 +3542,14 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Average Earnings excl. Bonus (3Mo/Yr)DEC</t>
+          <t>HMRC Payrolls ChangeJAN</t>
         </is>
       </c>
       <c r="D106" t="inlineStr"/>
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
-          <t>5.9%</t>
+          <t>-55.0K</t>
         </is>
       </c>
       <c r="G106" t="n">
@@ -3596,14 +3596,14 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>HMRC Payrolls ChangeJAN</t>
+          <t>Average Earnings excl. Bonus (3Mo/Yr)DEC</t>
         </is>
       </c>
       <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
-          <t>-55.0K</t>
+          <t>5.9%</t>
         </is>
       </c>
       <c r="G108" t="n">
@@ -3809,14 +3809,18 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>BoE Gov Bailey Speech</t>
+          <t>Labour Productivity QoQ PrelQ4</t>
         </is>
       </c>
       <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr"/>
-      <c r="F115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>-0.1%</t>
+        </is>
+      </c>
       <c r="G115" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="116">
@@ -3827,23 +3831,23 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>ZA</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Labour Productivity QoQ PrelQ4</t>
+          <t>Unemployment RateQ4</t>
         </is>
       </c>
       <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
-          <t>-0.1%</t>
+          <t>32.4%</t>
         </is>
       </c>
       <c r="G116" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="117">
@@ -3859,18 +3863,18 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Unemployment RateQ4</t>
+          <t>Unemployed PersonsQ4</t>
         </is>
       </c>
       <c r="D117" t="inlineStr"/>
       <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
-          <t>32.4%</t>
+          <t>8.1M</t>
         </is>
       </c>
       <c r="G117" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="118">
@@ -3881,23 +3885,19 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>ZA</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Unemployed PersonsQ4</t>
+          <t>BoE Gov Bailey Speech</t>
         </is>
       </c>
       <c r="D118" t="inlineStr"/>
       <c r="E118" t="inlineStr"/>
-      <c r="F118" t="inlineStr">
-        <is>
-          <t>8.1M</t>
-        </is>
-      </c>
+      <c r="F118" t="inlineStr"/>
       <c r="G118" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="119">
@@ -4595,22 +4595,22 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Machinery Orders YoYDEC</t>
+          <t>Imports YoYJAN</t>
         </is>
       </c>
       <c r="D145" t="inlineStr"/>
       <c r="E145" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>7.6%</t>
+          <t>2.0%</t>
         </is>
       </c>
       <c r="G145" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="146">
@@ -4626,22 +4626,22 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Imports YoYJAN</t>
+          <t>Machinery Orders MoMDEC</t>
         </is>
       </c>
       <c r="D146" t="inlineStr"/>
       <c r="E146" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>0.1%</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>2.0%</t>
+          <t>2.2%</t>
         </is>
       </c>
       <c r="G146" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="147">
@@ -4657,18 +4657,18 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Machinery Orders MoMDEC</t>
+          <t>Machinery Orders YoYDEC</t>
         </is>
       </c>
       <c r="D147" t="inlineStr"/>
       <c r="E147" t="inlineStr">
         <is>
-          <t>0.1%</t>
+          <t>6.9%</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>2.2%</t>
+          <t>7.6%</t>
         </is>
       </c>
       <c r="G147" t="n">
@@ -5306,18 +5306,18 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Lending Facility RateFEB</t>
+          <t>Deposit Facility RateFEB</t>
         </is>
       </c>
       <c r="D170" t="inlineStr"/>
       <c r="E170" t="inlineStr">
         <is>
-          <t>6.5%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>6.5%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="G170" t="n">
@@ -5337,18 +5337,18 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Deposit Facility RateFEB</t>
+          <t>Lending Facility RateFEB</t>
         </is>
       </c>
       <c r="D171" t="inlineStr"/>
       <c r="E171" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="G171" t="n">
@@ -5583,17 +5583,21 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>4-Year Treasury Gilt Auction</t>
+          <t>Current AccountDEC</t>
         </is>
       </c>
       <c r="D180" t="inlineStr"/>
       <c r="E180" t="inlineStr"/>
-      <c r="F180" t="inlineStr"/>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>€ 3780M</t>
+        </is>
+      </c>
       <c r="G180" t="n">
         <v>3</v>
       </c>
@@ -5606,21 +5610,17 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Current AccountDEC</t>
+          <t>4-Year Treasury Gilt Auction</t>
         </is>
       </c>
       <c r="D181" t="inlineStr"/>
       <c r="E181" t="inlineStr"/>
-      <c r="F181" t="inlineStr">
-        <is>
-          <t>€ 3780M</t>
-        </is>
-      </c>
+      <c r="F181" t="inlineStr"/>
       <c r="G181" t="n">
         <v>3</v>
       </c>
@@ -5899,18 +5899,18 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Housing StartsJAN</t>
+          <t>Building Permits PrelJAN</t>
         </is>
       </c>
       <c r="D193" t="inlineStr"/>
       <c r="E193" t="inlineStr">
         <is>
-          <t>1.39M</t>
+          <t>1.45M</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>1.35M</t>
+          <t>1.47M</t>
         </is>
       </c>
       <c r="G193" t="n">
@@ -5930,18 +5930,22 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Housing Starts MoMJAN</t>
+          <t>Housing StartsJAN</t>
         </is>
       </c>
       <c r="D194" t="inlineStr"/>
-      <c r="E194" t="inlineStr"/>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>1.39M</t>
+        </is>
+      </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>-9.0%</t>
+          <t>1.35M</t>
         </is>
       </c>
       <c r="G194" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="195">
@@ -5984,22 +5988,18 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Building Permits PrelJAN</t>
+          <t>Housing Starts MoMJAN</t>
         </is>
       </c>
       <c r="D196" t="inlineStr"/>
-      <c r="E196" t="inlineStr">
-        <is>
-          <t>1.45M</t>
-        </is>
-      </c>
+      <c r="E196" t="inlineStr"/>
       <c r="F196" t="inlineStr">
         <is>
-          <t>1.47M</t>
+          <t>-9.0%</t>
         </is>
       </c>
       <c r="G196" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="197">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Foreign Bond InvestmentFEB/15</t>
+          <t>Stock Investment by ForeignersFEB/15</t>
         </is>
       </c>
       <c r="D210" t="inlineStr"/>
@@ -6365,7 +6365,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Stock Investment by ForeignersFEB/15</t>
+          <t>Foreign Bond InvestmentFEB/15</t>
         </is>
       </c>
       <c r="D211" t="inlineStr"/>
@@ -6616,12 +6616,16 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>M2 Money Supply YoYJAN</t>
+          <t>Current AccountQ4</t>
         </is>
       </c>
       <c r="D220" t="inlineStr"/>
       <c r="E220" t="inlineStr"/>
-      <c r="F220" t="inlineStr"/>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>$ -0.6B</t>
+        </is>
+      </c>
       <c r="G220" t="n">
         <v>3</v>
       </c>
@@ -6634,21 +6638,17 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>Consumer ConfidenceJAN</t>
+          <t>M2 Money Supply YoYJAN</t>
         </is>
       </c>
       <c r="D221" t="inlineStr"/>
       <c r="E221" t="inlineStr"/>
-      <c r="F221" t="inlineStr">
-        <is>
-          <t>85.5</t>
-        </is>
-      </c>
+      <c r="F221" t="inlineStr"/>
       <c r="G221" t="n">
         <v>3</v>
       </c>
@@ -6661,19 +6661,19 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Current AccountQ4</t>
+          <t>Consumer ConfidenceJAN</t>
         </is>
       </c>
       <c r="D222" t="inlineStr"/>
       <c r="E222" t="inlineStr"/>
       <c r="F222" t="inlineStr">
         <is>
-          <t>$ -0.6B</t>
+          <t>85.5</t>
         </is>
       </c>
       <c r="G222" t="n">
@@ -6970,7 +6970,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>11-Year Index-Linked OAT Auction</t>
+          <t>6-Year Index-Linked OAT Auction</t>
         </is>
       </c>
       <c r="D234" t="inlineStr"/>
@@ -6988,19 +6988,27 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>18-Year Index-Linked OAT Auction</t>
+          <t>CBI Industrial Trends OrdersFEB</t>
         </is>
       </c>
       <c r="D235" t="inlineStr"/>
-      <c r="E235" t="inlineStr"/>
-      <c r="F235" t="inlineStr"/>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>-30</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>-25</t>
+        </is>
+      </c>
       <c r="G235" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="236">
@@ -7011,17 +7019,21 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>ZA</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>6-Year Index-Linked OAT Auction</t>
+          <t>Building Permits YoYDEC</t>
         </is>
       </c>
       <c r="D236" t="inlineStr"/>
       <c r="E236" t="inlineStr"/>
-      <c r="F236" t="inlineStr"/>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>18.0%</t>
+        </is>
+      </c>
       <c r="G236" t="n">
         <v>3</v>
       </c>
@@ -7057,21 +7069,17 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>ZA</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Building Permits YoYDEC</t>
+          <t>11-Year Index-Linked OAT Auction</t>
         </is>
       </c>
       <c r="D238" t="inlineStr"/>
       <c r="E238" t="inlineStr"/>
-      <c r="F238" t="inlineStr">
-        <is>
-          <t>18.0%</t>
-        </is>
-      </c>
+      <c r="F238" t="inlineStr"/>
       <c r="G238" t="n">
         <v>3</v>
       </c>
@@ -7084,27 +7092,19 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>CBI Industrial Trends OrdersFEB</t>
+          <t>18-Year Index-Linked OAT Auction</t>
         </is>
       </c>
       <c r="D239" t="inlineStr"/>
-      <c r="E239" t="inlineStr">
-        <is>
-          <t>-30</t>
-        </is>
-      </c>
-      <c r="F239" t="inlineStr">
-        <is>
-          <t>-25</t>
-        </is>
-      </c>
+      <c r="E239" t="inlineStr"/>
+      <c r="F239" t="inlineStr"/>
       <c r="G239" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="240">
@@ -7220,12 +7220,16 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Philly Fed CAPEX IndexFEB</t>
+          <t>Jobless Claims 4-week AverageFEB/15</t>
         </is>
       </c>
       <c r="D244" t="inlineStr"/>
       <c r="E244" t="inlineStr"/>
-      <c r="F244" t="inlineStr"/>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>219.0K</t>
+        </is>
+      </c>
       <c r="G244" t="n">
         <v>3</v>
       </c>
@@ -7238,21 +7242,17 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Raw Materials Prices MoMJAN</t>
+          <t>Philly Fed CAPEX IndexFEB</t>
         </is>
       </c>
       <c r="D245" t="inlineStr"/>
       <c r="E245" t="inlineStr"/>
-      <c r="F245" t="inlineStr">
-        <is>
-          <t>-0.2%</t>
-        </is>
-      </c>
+      <c r="F245" t="inlineStr"/>
       <c r="G245" t="n">
         <v>3</v>
       </c>
@@ -7270,12 +7270,16 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Philly Fed New OrdersFEB</t>
+          <t>Continuing Jobless ClaimsFEB/08</t>
         </is>
       </c>
       <c r="D246" t="inlineStr"/>
       <c r="E246" t="inlineStr"/>
-      <c r="F246" t="inlineStr"/>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>1879.0K</t>
+        </is>
+      </c>
       <c r="G246" t="n">
         <v>3</v>
       </c>
@@ -7293,16 +7297,12 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Jobless Claims 4-week AverageFEB/15</t>
+          <t>Philly Fed New OrdersFEB</t>
         </is>
       </c>
       <c r="D247" t="inlineStr"/>
       <c r="E247" t="inlineStr"/>
-      <c r="F247" t="inlineStr">
-        <is>
-          <t>219.0K</t>
-        </is>
-      </c>
+      <c r="F247" t="inlineStr"/>
       <c r="G247" t="n">
         <v>3</v>
       </c>
@@ -7366,18 +7366,22 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Continuing Jobless ClaimsFEB/08</t>
+          <t>Philadelphia Fed Manufacturing IndexFEB</t>
         </is>
       </c>
       <c r="D250" t="inlineStr"/>
-      <c r="E250" t="inlineStr"/>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>25.5</t>
+        </is>
+      </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>1879.0K</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G250" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="251">
@@ -7393,14 +7397,14 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>PPI MoMJAN</t>
+          <t>Raw Materials Prices YoYJAN</t>
         </is>
       </c>
       <c r="D251" t="inlineStr"/>
       <c r="E251" t="inlineStr"/>
       <c r="F251" t="inlineStr">
         <is>
-          <t>0.4%</t>
+          <t>10.0%</t>
         </is>
       </c>
       <c r="G251" t="n">
@@ -7415,27 +7419,23 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Initial Jobless ClaimsFEB/15</t>
+          <t>Raw Materials Prices MoMJAN</t>
         </is>
       </c>
       <c r="D252" t="inlineStr"/>
-      <c r="E252" t="inlineStr">
-        <is>
-          <t>216K</t>
-        </is>
-      </c>
+      <c r="E252" t="inlineStr"/>
       <c r="F252" t="inlineStr">
         <is>
-          <t>220.0K</t>
+          <t>-0.2%</t>
         </is>
       </c>
       <c r="G252" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="253">
@@ -7451,18 +7451,18 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>New Housing Price Index MoMJAN</t>
+          <t>PPI YoYJAN</t>
         </is>
       </c>
       <c r="D253" t="inlineStr"/>
       <c r="E253" t="inlineStr"/>
       <c r="F253" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>4.3%</t>
         </is>
       </c>
       <c r="G253" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="254">
@@ -7478,18 +7478,18 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>New Housing Price Index YoYJAN</t>
+          <t>PPI MoMJAN</t>
         </is>
       </c>
       <c r="D254" t="inlineStr"/>
       <c r="E254" t="inlineStr"/>
       <c r="F254" t="inlineStr">
         <is>
-          <t>0.2%</t>
+          <t>0.4%</t>
         </is>
       </c>
       <c r="G254" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="255">
@@ -7500,23 +7500,19 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Philadelphia Fed Manufacturing IndexFEB</t>
+          <t>New Housing Price Index YoYJAN</t>
         </is>
       </c>
       <c r="D255" t="inlineStr"/>
-      <c r="E255" t="inlineStr">
-        <is>
-          <t>25.5</t>
-        </is>
-      </c>
+      <c r="E255" t="inlineStr"/>
       <c r="F255" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>0.2%</t>
         </is>
       </c>
       <c r="G255" t="n">
@@ -7536,18 +7532,18 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>PPI YoYJAN</t>
+          <t>New Housing Price Index MoMJAN</t>
         </is>
       </c>
       <c r="D256" t="inlineStr"/>
       <c r="E256" t="inlineStr"/>
       <c r="F256" t="inlineStr">
         <is>
-          <t>4.3%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G256" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="257">
@@ -7558,23 +7554,27 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Raw Materials Prices YoYJAN</t>
+          <t>Initial Jobless ClaimsFEB/15</t>
         </is>
       </c>
       <c r="D257" t="inlineStr"/>
-      <c r="E257" t="inlineStr"/>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>216K</t>
+        </is>
+      </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>220.0K</t>
         </is>
       </c>
       <c r="G257" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="258">
@@ -7771,7 +7771,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>4-Week Bill Auction</t>
+          <t>8-Week Bill Auction</t>
         </is>
       </c>
       <c r="D265" t="inlineStr"/>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>8-Week Bill Auction</t>
+          <t>4-Week Bill Auction</t>
         </is>
       </c>
       <c r="D266" t="inlineStr"/>
@@ -7817,7 +7817,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>EIA Cushing Crude Oil Stocks ChangeFEB/14</t>
+          <t>EIA Distillate Stocks ChangeFEB/14</t>
         </is>
       </c>
       <c r="D267" t="inlineStr"/>
@@ -7840,7 +7840,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>EIA Heating Oil Stocks ChangeFEB/14</t>
+          <t>EIA Gasoline Production ChangeFEB/14</t>
         </is>
       </c>
       <c r="D268" t="inlineStr"/>
@@ -7863,7 +7863,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>EIA Refinery Crude Runs ChangeFEB/14</t>
+          <t>EIA Distillate Fuel Production ChangeFEB/14</t>
         </is>
       </c>
       <c r="D269" t="inlineStr"/>
@@ -7886,7 +7886,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>EIA Gasoline Production ChangeFEB/14</t>
+          <t>EIA Refinery Crude Runs ChangeFEB/14</t>
         </is>
       </c>
       <c r="D270" t="inlineStr"/>
@@ -7909,7 +7909,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>EIA Distillate Stocks ChangeFEB/14</t>
+          <t>EIA Heating Oil Stocks ChangeFEB/14</t>
         </is>
       </c>
       <c r="D271" t="inlineStr"/>
@@ -7932,7 +7932,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>EIA Distillate Fuel Production ChangeFEB/14</t>
+          <t>EIA Crude Oil Imports ChangeFEB/14</t>
         </is>
       </c>
       <c r="D272" t="inlineStr"/>
@@ -7955,7 +7955,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>EIA Crude Oil Imports ChangeFEB/14</t>
+          <t>EIA Cushing Crude Oil Stocks ChangeFEB/14</t>
         </is>
       </c>
       <c r="D273" t="inlineStr"/>
@@ -8207,21 +8207,17 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>S&amp;P Global Australia Manufacturing PMI FlashFEB</t>
+          <t>Fed Kugler Speech</t>
         </is>
       </c>
       <c r="D284" t="inlineStr"/>
       <c r="E284" t="inlineStr"/>
-      <c r="F284" t="inlineStr">
-        <is>
-          <t>49.9</t>
-        </is>
-      </c>
+      <c r="F284" t="inlineStr"/>
       <c r="G284" t="n">
         <v>2</v>
       </c>
@@ -8239,18 +8235,18 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>S&amp;P Global Australia Services PMI FlashFEB</t>
+          <t>S&amp;P Global Australia Composite PMI FlashFEB</t>
         </is>
       </c>
       <c r="D285" t="inlineStr"/>
       <c r="E285" t="inlineStr"/>
       <c r="F285" t="inlineStr">
         <is>
-          <t>51.3</t>
+          <t>50.6</t>
         </is>
       </c>
       <c r="G285" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="286">
@@ -8266,18 +8262,18 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>S&amp;P Global Australia Composite PMI FlashFEB</t>
+          <t>S&amp;P Global Australia Manufacturing PMI FlashFEB</t>
         </is>
       </c>
       <c r="D286" t="inlineStr"/>
       <c r="E286" t="inlineStr"/>
       <c r="F286" t="inlineStr">
         <is>
-          <t>50.6</t>
+          <t>49.9</t>
         </is>
       </c>
       <c r="G286" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="287">
@@ -8288,17 +8284,21 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Fed Kugler Speech</t>
+          <t>S&amp;P Global Australia Services PMI FlashFEB</t>
         </is>
       </c>
       <c r="D287" t="inlineStr"/>
       <c r="E287" t="inlineStr"/>
-      <c r="F287" t="inlineStr"/>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>51.3</t>
+        </is>
+      </c>
       <c r="G287" t="n">
         <v>2</v>
       </c>
@@ -8343,18 +8343,18 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Inflation Rate YoYJAN</t>
+          <t>Inflation Rate MoMJAN</t>
         </is>
       </c>
       <c r="D289" t="inlineStr"/>
       <c r="E289" t="inlineStr"/>
       <c r="F289" t="inlineStr">
         <is>
-          <t>3.7%</t>
+          <t>0.2%</t>
         </is>
       </c>
       <c r="G289" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="290">
@@ -8370,22 +8370,18 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>Core Inflation Rate YoYJAN</t>
+          <t>Inflation Rate YoYJAN</t>
         </is>
       </c>
       <c r="D290" t="inlineStr"/>
-      <c r="E290" t="inlineStr">
-        <is>
-          <t>3.1%</t>
-        </is>
-      </c>
+      <c r="E290" t="inlineStr"/>
       <c r="F290" t="inlineStr">
         <is>
-          <t>3.2%</t>
+          <t>3.7%</t>
         </is>
       </c>
       <c r="G290" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="291">
@@ -8401,18 +8397,22 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Inflation Rate Ex-Food and Energy YoYJAN</t>
+          <t>Core Inflation Rate YoYJAN</t>
         </is>
       </c>
       <c r="D291" t="inlineStr"/>
-      <c r="E291" t="inlineStr"/>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>3.1%</t>
+        </is>
+      </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>2.6%</t>
+          <t>3.2%</t>
         </is>
       </c>
       <c r="G291" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="292">
@@ -8428,14 +8428,14 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Inflation Rate MoMJAN</t>
+          <t>Inflation Rate Ex-Food and Energy YoYJAN</t>
         </is>
       </c>
       <c r="D292" t="inlineStr"/>
       <c r="E292" t="inlineStr"/>
       <c r="F292" t="inlineStr">
         <is>
-          <t>0.2%</t>
+          <t>2.6%</t>
         </is>
       </c>
       <c r="G292" t="n">
@@ -8486,18 +8486,22 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Jibun Bank Composite PMI FlashFEB</t>
+          <t>Jibun Bank Manufacturing PMI FlashFEB</t>
         </is>
       </c>
       <c r="D294" t="inlineStr"/>
-      <c r="E294" t="inlineStr"/>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>51.5</t>
+          <t>49.6</t>
         </is>
       </c>
       <c r="G294" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="295">
@@ -8540,22 +8544,18 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Jibun Bank Manufacturing PMI FlashFEB</t>
+          <t>Jibun Bank Composite PMI FlashFEB</t>
         </is>
       </c>
       <c r="D296" t="inlineStr"/>
-      <c r="E296" t="inlineStr">
-        <is>
-          <t>49</t>
-        </is>
-      </c>
+      <c r="E296" t="inlineStr"/>
       <c r="F296" t="inlineStr">
         <is>
-          <t>49.6</t>
+          <t>51.5</t>
         </is>
       </c>
       <c r="G296" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="297">
@@ -8612,17 +8612,21 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>3-Month Bill Auction</t>
+          <t>Central Government DebtJAN</t>
         </is>
       </c>
       <c r="D299" t="inlineStr"/>
       <c r="E299" t="inlineStr"/>
-      <c r="F299" t="inlineStr"/>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>TRY 9.4T</t>
+        </is>
+      </c>
       <c r="G299" t="n">
         <v>3</v>
       </c>
@@ -8635,21 +8639,17 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Central Government DebtJAN</t>
+          <t>10-Year NTN-F Auction</t>
         </is>
       </c>
       <c r="D300" t="inlineStr"/>
       <c r="E300" t="inlineStr"/>
-      <c r="F300" t="inlineStr">
-        <is>
-          <t>TRY 9.4T</t>
-        </is>
-      </c>
+      <c r="F300" t="inlineStr"/>
       <c r="G300" t="n">
         <v>3</v>
       </c>
@@ -8662,12 +8662,12 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>10-Year NTN-F Auction</t>
+          <t>3-Month Bill Auction</t>
         </is>
       </c>
       <c r="D301" t="inlineStr"/>
@@ -8771,18 +8771,22 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Retail Sales ex Fuel YoYJAN</t>
+          <t>Retail Sales MoMJAN</t>
         </is>
       </c>
       <c r="D305" t="inlineStr"/>
-      <c r="E305" t="inlineStr"/>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>0.3%</t>
+        </is>
+      </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>0.2%</t>
         </is>
       </c>
       <c r="G305" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="306">
@@ -8798,22 +8802,18 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>Retail Sales MoMJAN</t>
+          <t>Retail Sales YoYJAN</t>
         </is>
       </c>
       <c r="D306" t="inlineStr"/>
-      <c r="E306" t="inlineStr">
-        <is>
-          <t>0.3%</t>
-        </is>
-      </c>
+      <c r="E306" t="inlineStr"/>
       <c r="F306" t="inlineStr">
         <is>
-          <t>0.2%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="G306" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="307">
@@ -8829,18 +8829,22 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>Retail Sales YoYJAN</t>
+          <t>Public Sector Net Borrowing Ex BanksJAN</t>
         </is>
       </c>
       <c r="D307" t="inlineStr"/>
-      <c r="E307" t="inlineStr"/>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>£20.5B</t>
+        </is>
+      </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>£19.0B</t>
         </is>
       </c>
       <c r="G307" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="308">
@@ -8856,18 +8860,14 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>Public Sector Net Borrowing Ex BanksJAN</t>
+          <t>Retail Sales ex Fuel MoMJAN</t>
         </is>
       </c>
       <c r="D308" t="inlineStr"/>
-      <c r="E308" t="inlineStr">
-        <is>
-          <t>£20.5B</t>
-        </is>
-      </c>
+      <c r="E308" t="inlineStr"/>
       <c r="F308" t="inlineStr">
         <is>
-          <t>£19.0B</t>
+          <t>0.3%</t>
         </is>
       </c>
       <c r="G308" t="n">
@@ -8887,14 +8887,14 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Retail Sales ex Fuel MoMJAN</t>
+          <t>Retail Sales ex Fuel YoYJAN</t>
         </is>
       </c>
       <c r="D309" t="inlineStr"/>
       <c r="E309" t="inlineStr"/>
       <c r="F309" t="inlineStr">
         <is>
-          <t>0.3%</t>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="G309" t="n">
@@ -8914,18 +8914,18 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>Business ConfidenceFEB</t>
+          <t>Business Climate IndicatorFEB</t>
         </is>
       </c>
       <c r="D310" t="inlineStr"/>
       <c r="E310" t="inlineStr"/>
       <c r="F310" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>92</t>
         </is>
       </c>
       <c r="G310" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="311">
@@ -8941,18 +8941,18 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>Business Climate IndicatorFEB</t>
+          <t>Business ConfidenceFEB</t>
         </is>
       </c>
       <c r="D311" t="inlineStr"/>
       <c r="E311" t="inlineStr"/>
       <c r="F311" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>94</t>
         </is>
       </c>
       <c r="G311" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="312">
@@ -9200,22 +9200,22 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>Inflation Rate MoM FinalJAN</t>
+          <t>Harmonised Inflation Rate MoM FinalJAN</t>
         </is>
       </c>
       <c r="D320" t="inlineStr"/>
       <c r="E320" t="inlineStr">
         <is>
-          <t>0.6%</t>
+          <t>-0.7%</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>0.6%</t>
+          <t>-0.7%</t>
         </is>
       </c>
       <c r="G320" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="321">
@@ -9231,22 +9231,22 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>Harmonised Inflation Rate MoM FinalJAN</t>
+          <t>Inflation Rate YoY FinalJAN</t>
         </is>
       </c>
       <c r="D321" t="inlineStr"/>
       <c r="E321" t="inlineStr">
         <is>
-          <t>-0.7%</t>
+          <t>1.5%</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>-0.7%</t>
+          <t>1.5%</t>
         </is>
       </c>
       <c r="G321" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="322">
@@ -9262,18 +9262,18 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Inflation Rate YoY FinalJAN</t>
+          <t>Inflation Rate MoM FinalJAN</t>
         </is>
       </c>
       <c r="D322" t="inlineStr"/>
       <c r="E322" t="inlineStr">
         <is>
-          <t>1.5%</t>
+          <t>0.6%</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>1.5%</t>
+          <t>0.6%</t>
         </is>
       </c>
       <c r="G322" t="n">
@@ -9517,14 +9517,14 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Economic Activity MoMDEC</t>
+          <t>Economic Activity YoYDEC</t>
         </is>
       </c>
       <c r="D331" t="inlineStr"/>
       <c r="E331" t="inlineStr"/>
       <c r="F331" t="inlineStr">
         <is>
-          <t>0.5%</t>
+          <t>2%</t>
         </is>
       </c>
       <c r="G331" t="n">
@@ -9544,18 +9544,22 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Economic Activity YoYDEC</t>
+          <t>GDP Growth Rate YoY FinalQ4</t>
         </is>
       </c>
       <c r="D332" t="inlineStr"/>
-      <c r="E332" t="inlineStr"/>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>0.6%</t>
+        </is>
+      </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>2%</t>
+          <t>0.6%</t>
         </is>
       </c>
       <c r="G332" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="333">
@@ -9571,22 +9575,18 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>GDP Growth Rate YoY FinalQ4</t>
+          <t>Economic Activity MoMDEC</t>
         </is>
       </c>
       <c r="D333" t="inlineStr"/>
-      <c r="E333" t="inlineStr">
-        <is>
-          <t>0.6%</t>
-        </is>
-      </c>
+      <c r="E333" t="inlineStr"/>
       <c r="F333" t="inlineStr">
         <is>
-          <t>0.6%</t>
+          <t>0.5%</t>
         </is>
       </c>
       <c r="G333" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="334">
@@ -9772,7 +9772,7 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>S&amp;P Global Services PMI FlashFEB</t>
+          <t>S&amp;P Global Composite PMI FlashFEB</t>
         </is>
       </c>
       <c r="D340" t="inlineStr"/>
@@ -9799,14 +9799,14 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>S&amp;P Global Composite PMI FlashFEB</t>
+          <t>S&amp;P Global Manufacturing PMI FlashFEB</t>
         </is>
       </c>
       <c r="D341" t="inlineStr"/>
       <c r="E341" t="inlineStr"/>
       <c r="F341" t="inlineStr">
         <is>
-          <t>52.7</t>
+          <t>51.3</t>
         </is>
       </c>
       <c r="G341" t="n">
@@ -9826,14 +9826,14 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>S&amp;P Global Manufacturing PMI FlashFEB</t>
+          <t>S&amp;P Global Services PMI FlashFEB</t>
         </is>
       </c>
       <c r="D342" t="inlineStr"/>
       <c r="E342" t="inlineStr"/>
       <c r="F342" t="inlineStr">
         <is>
-          <t>51.3</t>
+          <t>52.7</t>
         </is>
       </c>
       <c r="G342" t="n">
@@ -9853,18 +9853,18 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>Michigan Consumer Expectations FinalFEB</t>
+          <t>Michigan Current Conditions FinalFEB</t>
         </is>
       </c>
       <c r="D343" t="inlineStr"/>
       <c r="E343" t="inlineStr">
         <is>
-          <t>67.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>67.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="G343" t="n">
@@ -9915,18 +9915,18 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>Michigan Current Conditions FinalFEB</t>
+          <t>Michigan Consumer Expectations FinalFEB</t>
         </is>
       </c>
       <c r="D345" t="inlineStr"/>
       <c r="E345" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>67.3</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>67.3</t>
         </is>
       </c>
       <c r="G345" t="n">
@@ -9977,14 +9977,18 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>Existing Home Sales MoMJAN</t>
+          <t>Michigan Consumer Sentiment FinalFEB</t>
         </is>
       </c>
       <c r="D347" t="inlineStr"/>
-      <c r="E347" t="inlineStr"/>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>67.8</t>
+        </is>
+      </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>-1.7%</t>
+          <t>67.8</t>
         </is>
       </c>
       <c r="G347" t="n">
@@ -10004,18 +10008,14 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>Michigan Consumer Sentiment FinalFEB</t>
+          <t>Existing Home Sales MoMJAN</t>
         </is>
       </c>
       <c r="D348" t="inlineStr"/>
-      <c r="E348" t="inlineStr">
-        <is>
-          <t>67.8</t>
-        </is>
-      </c>
+      <c r="E348" t="inlineStr"/>
       <c r="F348" t="inlineStr">
         <is>
-          <t>67.8</t>
+          <t>-1.7%</t>
         </is>
       </c>
       <c r="G348" t="n">
@@ -10379,18 +10379,18 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>Ifo ExpectationsFEB</t>
+          <t>Ifo Business ClimateFEB</t>
         </is>
       </c>
       <c r="D363" t="inlineStr"/>
       <c r="E363" t="inlineStr"/>
       <c r="F363" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>84</t>
         </is>
       </c>
       <c r="G363" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="364">
@@ -10406,18 +10406,18 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>Ifo Business ClimateFEB</t>
+          <t>Ifo Current ConditionsFEB</t>
         </is>
       </c>
       <c r="D364" t="inlineStr"/>
       <c r="E364" t="inlineStr"/>
       <c r="F364" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85.1</t>
         </is>
       </c>
       <c r="G364" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="365">
@@ -10433,14 +10433,14 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>Ifo Current ConditionsFEB</t>
+          <t>Ifo ExpectationsFEB</t>
         </is>
       </c>
       <c r="D365" t="inlineStr"/>
       <c r="E365" t="inlineStr"/>
       <c r="F365" t="inlineStr">
         <is>
-          <t>85.1</t>
+          <t>83</t>
         </is>
       </c>
       <c r="G365" t="n">
@@ -10460,18 +10460,18 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>Inflation Rate MoM FinalJAN</t>
+          <t>CPI FinalJAN</t>
         </is>
       </c>
       <c r="D366" t="inlineStr"/>
       <c r="E366" t="inlineStr">
         <is>
-          <t>-0.3%</t>
+          <t>126.71</t>
         </is>
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>-0.3%</t>
+          <t>126.71</t>
         </is>
       </c>
       <c r="G366" t="n">
@@ -10491,18 +10491,18 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>CPI FinalJAN</t>
+          <t>Inflation Rate MoM FinalJAN</t>
         </is>
       </c>
       <c r="D367" t="inlineStr"/>
       <c r="E367" t="inlineStr">
         <is>
-          <t>126.71</t>
+          <t>-0.3%</t>
         </is>
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t>126.71</t>
+          <t>-0.3%</t>
         </is>
       </c>
       <c r="G367" t="n">
@@ -10676,7 +10676,7 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>Mid-month Inflation Rate MoMFEB</t>
+          <t>Mid-month Inflation Rate YoYFEB</t>
         </is>
       </c>
       <c r="D374" t="inlineStr"/>
@@ -10745,7 +10745,7 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>Mid-month Inflation Rate YoYFEB</t>
+          <t>Mid-month Inflation Rate MoMFEB</t>
         </is>
       </c>
       <c r="D377" t="inlineStr"/>
@@ -11139,6 +11139,118 @@
         <v>3</v>
       </c>
     </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2025-02-25 02:00:00-05:00</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>GDP Growth Rate QoQ FinalQ4</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr"/>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>-0.2%</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>-0.2%</t>
+        </is>
+      </c>
+      <c r="G394" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2025-02-25 02:00:00-05:00</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>GDP Growth Rate YoY FinalQ4</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr"/>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>-0.2%</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>-0.2%</t>
+        </is>
+      </c>
+      <c r="G395" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2025-02-25 02:00:00-05:00</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>New Car Registrations YoYJAN</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr"/>
+      <c r="E396" t="inlineStr"/>
+      <c r="F396" t="inlineStr"/>
+      <c r="G396" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2025-02-25 02:00:00-05:00</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>ZA</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Leading Business Cycle Indicator MoMDEC</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr"/>
+      <c r="E397" t="inlineStr"/>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>0.3%</t>
+        </is>
+      </c>
+      <c r="G397" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>